<commit_message>
Now using Raymer empty weight calculation so cost is a function of geometry. Fixed struct2array. Added fall back if excel is open
</commit_message>
<xml_diff>
--- a/Sizing/concepts_tabulations_template.xlsx
+++ b/Sizing/concepts_tabulations_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfile\Documents\MyDocuments\CODING\GitWorkingDirectory\team10aiaa\Sizing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{439DC1FD-7780-4245-882F-C781C3C0B8A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7EE4D053-B444-404A-B4A4-9591ACFAEF25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="89">
   <si>
     <t>Deliverable</t>
   </si>
@@ -92,9 +92,6 @@
     <t>Empty Weight [lb]</t>
   </si>
   <si>
-    <t>MTOW will be computed from this</t>
-  </si>
-  <si>
     <t>LE Sweep [deg]</t>
   </si>
   <si>
@@ -164,15 +161,6 @@
     <t>700nm Strike Mission Fuel Remaining [lb]</t>
   </si>
   <si>
-    <t>Combat Mission Max Range [nm]</t>
-  </si>
-  <si>
-    <t>Strike Mission Max Range [nm]</t>
-  </si>
-  <si>
-    <t>Ferry Mission Max Range [nm]</t>
-  </si>
-  <si>
     <t>Max Wing Loading [N/m2]</t>
   </si>
   <si>
@@ -290,7 +278,31 @@
     <t>FA-18E Sized</t>
   </si>
   <si>
-    <t>X VTAIL MAC [m]</t>
+    <t>Combat Mission Max Radius [nm]</t>
+  </si>
+  <si>
+    <t>Strike Mission Max Radius [nm]</t>
+  </si>
+  <si>
+    <t>Ferry Mission Max Radius [nm]</t>
+  </si>
+  <si>
+    <t>Whatever is remaining in the weight</t>
+  </si>
+  <si>
+    <t>Computed using raymer</t>
+  </si>
+  <si>
+    <t>Folded Span [ft]</t>
+  </si>
+  <si>
+    <t>Folded Height [ft]</t>
+  </si>
+  <si>
+    <t>18.5ft Fold Height Limit</t>
+  </si>
+  <si>
+    <t>35ft Fold Limit</t>
   </si>
 </sst>
 </file>
@@ -847,18 +859,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2919600B-FD59-4F7A-AAA3-223AE9D885EC}">
-  <dimension ref="A1:L55"/>
+  <dimension ref="A1:L58"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="37.88671875" customWidth="1"/>
-    <col min="2" max="2" width="10.5546875" customWidth="1"/>
-    <col min="3" max="3" width="12.33203125" customWidth="1"/>
-    <col min="4" max="5" width="4.77734375" customWidth="1"/>
-    <col min="6" max="8" width="9.6640625" customWidth="1"/>
-    <col min="9" max="9" width="10.5546875" customWidth="1"/>
-    <col min="10" max="10" width="9.6640625" customWidth="1"/>
-    <col min="11" max="11" width="10.5546875" customWidth="1"/>
-    <col min="12" max="12" width="99.88671875" customWidth="1"/>
+    <col min="1" max="1" width="38.77734375" customWidth="1"/>
+    <col min="2" max="10" width="11.88671875" customWidth="1"/>
+    <col min="11" max="11" width="10.44140625" customWidth="1"/>
+    <col min="12" max="12" width="106.77734375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -866,13 +873,13 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>8</v>
@@ -881,7 +888,7 @@
         <v>1</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>2</v>
@@ -893,7 +900,7 @@
         <v>4</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="L1" s="6" t="s">
         <v>7</v>
@@ -917,7 +924,7 @@
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="B3" s="11"/>
       <c r="C3" s="11"/>
@@ -930,12 +937,12 @@
       <c r="J3" s="13"/>
       <c r="K3" s="13"/>
       <c r="L3" s="8" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A4" s="5" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="B4" s="11"/>
       <c r="C4" s="11"/>
@@ -948,12 +955,12 @@
       <c r="J4" s="13"/>
       <c r="K4" s="13"/>
       <c r="L4" s="8" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A5" s="5" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B5" s="11"/>
       <c r="C5" s="11"/>
@@ -966,12 +973,12 @@
       <c r="J5" s="13"/>
       <c r="K5" s="13"/>
       <c r="L5" s="8" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A6" s="5" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B6" s="11"/>
       <c r="C6" s="11"/>
@@ -984,12 +991,12 @@
       <c r="J6" s="13"/>
       <c r="K6" s="13"/>
       <c r="L6" s="8" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B7" s="11"/>
       <c r="C7" s="11"/>
@@ -1002,12 +1009,12 @@
       <c r="J7" s="13"/>
       <c r="K7" s="13"/>
       <c r="L7" s="8" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A8" s="5" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="B8" s="11"/>
       <c r="C8" s="11"/>
@@ -1020,12 +1027,12 @@
       <c r="J8" s="13"/>
       <c r="K8" s="13"/>
       <c r="L8" s="8" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A9" s="5" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B9" s="11"/>
       <c r="C9" s="11"/>
@@ -1041,7 +1048,7 @@
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A10" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B10" s="11"/>
       <c r="C10" s="11"/>
@@ -1057,7 +1064,7 @@
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A11" s="5" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="B11" s="11"/>
       <c r="C11" s="11"/>
@@ -1073,7 +1080,7 @@
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A12" s="5" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B12" s="11"/>
       <c r="C12" s="11"/>
@@ -1089,7 +1096,7 @@
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A13" s="5" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="B13" s="11"/>
       <c r="C13" s="11"/>
@@ -1105,7 +1112,7 @@
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A14" s="5" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="B14" s="11"/>
       <c r="C14" s="11"/>
@@ -1118,12 +1125,12 @@
       <c r="J14" s="12"/>
       <c r="K14" s="12"/>
       <c r="L14" s="9" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A15" s="5" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="B15" s="11"/>
       <c r="C15" s="11"/>
@@ -1136,12 +1143,12 @@
       <c r="J15" s="12"/>
       <c r="K15" s="12"/>
       <c r="L15" s="9" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A16" s="5" t="s">
-        <v>42</v>
+        <v>80</v>
       </c>
       <c r="B16" s="11"/>
       <c r="C16" s="11"/>
@@ -1157,7 +1164,7 @@
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A17" s="5" t="s">
-        <v>43</v>
+        <v>81</v>
       </c>
       <c r="B17" s="11"/>
       <c r="C17" s="11"/>
@@ -1173,7 +1180,7 @@
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A18" s="5" t="s">
-        <v>44</v>
+        <v>82</v>
       </c>
       <c r="B18" s="11"/>
       <c r="C18" s="11"/>
@@ -1189,7 +1196,7 @@
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A19" s="5" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B19" s="11"/>
       <c r="C19" s="11"/>
@@ -1205,7 +1212,7 @@
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A20" s="5" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B20" s="11"/>
       <c r="C20" s="11"/>
@@ -1221,7 +1228,7 @@
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A21" s="5" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="B21" s="11"/>
       <c r="C21" s="11"/>
@@ -1234,12 +1241,12 @@
       <c r="J21" s="12"/>
       <c r="K21" s="12"/>
       <c r="L21" s="9" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A22" s="5" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="B22" s="11"/>
       <c r="C22" s="11"/>
@@ -1252,7 +1259,7 @@
       <c r="J22" s="12"/>
       <c r="K22" s="12"/>
       <c r="L22" s="9" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.3">
@@ -1270,12 +1277,12 @@
       <c r="J23" s="12"/>
       <c r="K23" s="12"/>
       <c r="L23" s="9" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A24" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B24" s="15"/>
       <c r="C24" s="15"/>
@@ -1363,7 +1370,7 @@
     </row>
     <row r="29" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A29" s="5" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
       <c r="B29" s="11"/>
       <c r="C29" s="11"/>
@@ -1375,13 +1382,11 @@
       <c r="I29" s="12"/>
       <c r="J29" s="12"/>
       <c r="K29" s="12"/>
-      <c r="L29" s="9" t="s">
-        <v>18</v>
-      </c>
+      <c r="L29" s="9"/>
     </row>
     <row r="30" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A30" s="5" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B30" s="11"/>
       <c r="C30" s="11"/>
@@ -1394,12 +1399,12 @@
       <c r="J30" s="12"/>
       <c r="K30" s="12"/>
       <c r="L30" s="9" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="31" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A31" s="5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B31" s="11"/>
       <c r="C31" s="11"/>
@@ -1415,7 +1420,7 @@
     </row>
     <row r="32" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A32" s="5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B32" s="11"/>
       <c r="C32" s="11"/>
@@ -1428,12 +1433,12 @@
       <c r="J32" s="12"/>
       <c r="K32" s="12"/>
       <c r="L32" s="9" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="33" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A33" s="5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B33" s="11"/>
       <c r="C33" s="11"/>
@@ -1446,12 +1451,12 @@
       <c r="J33" s="12"/>
       <c r="K33" s="12"/>
       <c r="L33" s="9" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="34" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A34" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B34" s="11"/>
       <c r="C34" s="11"/>
@@ -1467,7 +1472,7 @@
     </row>
     <row r="35" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A35" s="5" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="B35" s="11"/>
       <c r="C35" s="11"/>
@@ -1480,12 +1485,12 @@
       <c r="J35" s="12"/>
       <c r="K35" s="12"/>
       <c r="L35" s="9" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
     </row>
     <row r="36" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A36" s="5" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B36" s="11"/>
       <c r="C36" s="11"/>
@@ -1498,12 +1503,12 @@
       <c r="J36" s="12"/>
       <c r="K36" s="12"/>
       <c r="L36" s="9" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="37" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A37" s="5" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="B37" s="11"/>
       <c r="C37" s="11"/>
@@ -1519,7 +1524,7 @@
     </row>
     <row r="38" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A38" s="4" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="B38" s="15"/>
       <c r="C38" s="15"/>
@@ -1538,36 +1543,40 @@
         <v>48</v>
       </c>
       <c r="B39" s="11"/>
-      <c r="C39" s="11"/>
-      <c r="D39" s="11"/>
-      <c r="E39" s="11"/>
-      <c r="F39" s="12"/>
-      <c r="G39" s="12"/>
-      <c r="H39" s="12"/>
-      <c r="I39" s="12"/>
+      <c r="C39" s="14"/>
+      <c r="D39" s="14"/>
+      <c r="E39" s="14"/>
+      <c r="F39" s="13"/>
+      <c r="G39" s="13"/>
+      <c r="H39" s="13"/>
+      <c r="I39" s="13"/>
       <c r="J39" s="12"/>
       <c r="K39" s="12"/>
-      <c r="L39" s="9"/>
+      <c r="L39" s="9" t="s">
+        <v>83</v>
+      </c>
     </row>
     <row r="40" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A40" s="5" t="s">
-        <v>52</v>
+        <v>17</v>
       </c>
       <c r="B40" s="11"/>
-      <c r="C40" s="14"/>
-      <c r="D40" s="14"/>
-      <c r="E40" s="14"/>
-      <c r="F40" s="13"/>
-      <c r="G40" s="13"/>
-      <c r="H40" s="13"/>
-      <c r="I40" s="13"/>
+      <c r="C40" s="11"/>
+      <c r="D40" s="11"/>
+      <c r="E40" s="11"/>
+      <c r="F40" s="12"/>
+      <c r="G40" s="12"/>
+      <c r="H40" s="12"/>
+      <c r="I40" s="12"/>
       <c r="J40" s="12"/>
       <c r="K40" s="12"/>
-      <c r="L40" s="9"/>
+      <c r="L40" s="9" t="s">
+        <v>84</v>
+      </c>
     </row>
     <row r="41" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A41" s="5" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B41" s="11"/>
       <c r="C41" s="14"/>
@@ -1583,7 +1592,7 @@
     </row>
     <row r="42" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A42" s="5" t="s">
-        <v>49</v>
+        <v>86</v>
       </c>
       <c r="B42" s="11"/>
       <c r="C42" s="14"/>
@@ -1599,7 +1608,7 @@
     </row>
     <row r="43" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A43" s="5" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="B43" s="11"/>
       <c r="C43" s="14"/>
@@ -1615,7 +1624,7 @@
     </row>
     <row r="44" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A44" s="5" t="s">
-        <v>54</v>
+        <v>46</v>
       </c>
       <c r="B44" s="11"/>
       <c r="C44" s="14"/>
@@ -1631,7 +1640,7 @@
     </row>
     <row r="45" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A45" s="5" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="B45" s="11"/>
       <c r="C45" s="14"/>
@@ -1647,7 +1656,7 @@
     </row>
     <row r="46" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A46" s="5" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="B46" s="11"/>
       <c r="C46" s="14"/>
@@ -1662,58 +1671,58 @@
       <c r="L46" s="9"/>
     </row>
     <row r="47" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A47" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="B47" s="15"/>
-      <c r="C47" s="15"/>
-      <c r="D47" s="15"/>
-      <c r="E47" s="15"/>
-      <c r="F47" s="15"/>
-      <c r="G47" s="15"/>
-      <c r="H47" s="15"/>
-      <c r="I47" s="15"/>
-      <c r="J47" s="15"/>
-      <c r="K47" s="15"/>
-      <c r="L47" s="10"/>
+      <c r="A47" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="B47" s="11"/>
+      <c r="C47" s="14"/>
+      <c r="D47" s="14"/>
+      <c r="E47" s="14"/>
+      <c r="F47" s="13"/>
+      <c r="G47" s="13"/>
+      <c r="H47" s="13"/>
+      <c r="I47" s="13"/>
+      <c r="J47" s="12"/>
+      <c r="K47" s="12"/>
+      <c r="L47" s="9"/>
     </row>
     <row r="48" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A48" s="5" t="s">
-        <v>68</v>
-      </c>
-      <c r="B48" s="11"/>
-      <c r="C48" s="11"/>
-      <c r="D48" s="11"/>
-      <c r="E48" s="11"/>
-      <c r="F48" s="12"/>
-      <c r="G48" s="12"/>
-      <c r="H48" s="12"/>
-      <c r="I48" s="12"/>
-      <c r="J48" s="12"/>
-      <c r="K48" s="12"/>
-      <c r="L48" s="9" t="s">
-        <v>70</v>
-      </c>
+      <c r="A48" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="B48" s="15"/>
+      <c r="C48" s="15"/>
+      <c r="D48" s="15"/>
+      <c r="E48" s="15"/>
+      <c r="F48" s="15"/>
+      <c r="G48" s="15"/>
+      <c r="H48" s="15"/>
+      <c r="I48" s="15"/>
+      <c r="J48" s="15"/>
+      <c r="K48" s="15"/>
+      <c r="L48" s="10"/>
     </row>
     <row r="49" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A49" s="5" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="B49" s="11"/>
-      <c r="C49" s="14"/>
-      <c r="D49" s="14"/>
-      <c r="E49" s="14"/>
-      <c r="F49" s="13"/>
-      <c r="G49" s="13"/>
-      <c r="H49" s="13"/>
-      <c r="I49" s="13"/>
+      <c r="C49" s="11"/>
+      <c r="D49" s="11"/>
+      <c r="E49" s="11"/>
+      <c r="F49" s="12"/>
+      <c r="G49" s="12"/>
+      <c r="H49" s="12"/>
+      <c r="I49" s="12"/>
       <c r="J49" s="12"/>
       <c r="K49" s="12"/>
-      <c r="L49" s="9"/>
+      <c r="L49" s="9" t="s">
+        <v>66</v>
+      </c>
     </row>
     <row r="50" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A50" s="5" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="B50" s="11"/>
       <c r="C50" s="14"/>
@@ -1729,7 +1738,7 @@
     </row>
     <row r="51" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A51" s="5" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="B51" s="11"/>
       <c r="C51" s="14"/>
@@ -1745,7 +1754,7 @@
     </row>
     <row r="52" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A52" s="5" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="B52" s="11"/>
       <c r="C52" s="14"/>
@@ -1761,7 +1770,7 @@
     </row>
     <row r="53" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A53" s="5" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="B53" s="11"/>
       <c r="C53" s="14"/>
@@ -1777,7 +1786,7 @@
     </row>
     <row r="54" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A54" s="5" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="B54" s="11"/>
       <c r="C54" s="14"/>
@@ -1793,7 +1802,7 @@
     </row>
     <row r="55" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A55" s="5" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="B55" s="11"/>
       <c r="C55" s="14"/>
@@ -1807,6 +1816,54 @@
       <c r="K55" s="12"/>
       <c r="L55" s="9"/>
     </row>
+    <row r="56" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A56" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="B56" s="11"/>
+      <c r="C56" s="14"/>
+      <c r="D56" s="14"/>
+      <c r="E56" s="14"/>
+      <c r="F56" s="13"/>
+      <c r="G56" s="13"/>
+      <c r="H56" s="13"/>
+      <c r="I56" s="13"/>
+      <c r="J56" s="12"/>
+      <c r="K56" s="12"/>
+      <c r="L56" s="9"/>
+    </row>
+    <row r="57" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A57" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="B57" s="11"/>
+      <c r="C57" s="14"/>
+      <c r="D57" s="14"/>
+      <c r="E57" s="14"/>
+      <c r="F57" s="13"/>
+      <c r="G57" s="13"/>
+      <c r="H57" s="13"/>
+      <c r="I57" s="13"/>
+      <c r="J57" s="12"/>
+      <c r="K57" s="12"/>
+      <c r="L57" s="9"/>
+    </row>
+    <row r="58" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A58" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="B58" s="11"/>
+      <c r="C58" s="14"/>
+      <c r="D58" s="14"/>
+      <c r="E58" s="14"/>
+      <c r="F58" s="13"/>
+      <c r="G58" s="13"/>
+      <c r="H58" s="13"/>
+      <c r="I58" s="13"/>
+      <c r="J58" s="12"/>
+      <c r="K58" s="12"/>
+      <c r="L58" s="9"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -1814,25 +1871,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f38bd768-81b4-450c-b73d-1a8fa3ba2722">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100841FCFF63B2DEE4FAB3ABDCB2B58E191" ma:contentTypeVersion="9" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="6537ae6c172b48d8001feb3057ef3193">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="f38bd768-81b4-450c-b73d-1a8fa3ba2722" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="e79d1da23033c2d9c1658a7b9c3763cb" ns2:_="">
     <xsd:import namespace="f38bd768-81b4-450c-b73d-1a8fa3ba2722"/>
@@ -2004,10 +2042,39 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f38bd768-81b4-450c-b73d-1a8fa3ba2722">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9162A322-41FC-4C0D-9942-C36B749F2613}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A0D3B35F-2651-4930-8D88-666C35501CF8}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="f38bd768-81b4-450c-b73d-1a8fa3ba2722"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -2023,19 +2090,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A0D3B35F-2651-4930-8D88-666C35501CF8}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9162A322-41FC-4C0D-9942-C36B749F2613}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="f38bd768-81b4-450c-b73d-1a8fa3ba2722"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Stability improvements and Liams rows
</commit_message>
<xml_diff>
--- a/Sizing/concepts_tabulations_template.xlsx
+++ b/Sizing/concepts_tabulations_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfile\Documents\MyDocuments\CODING\GitWorkingDirectory\team10aiaa\Sizing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{007308E2-E747-47EA-8F6F-F4656DD73D08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A629E1F0-03BC-4697-A28C-E4EA34D468C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="97">
   <si>
     <t>Deliverable</t>
   </si>
@@ -315,6 +315,18 @@
   </si>
   <si>
     <t>Hor Stab Planform Area [m2]</t>
+  </si>
+  <si>
+    <t>Hor Stab Aspect Ratio</t>
+  </si>
+  <si>
+    <t>Hor Stab Taper Ratio</t>
+  </si>
+  <si>
+    <t>Hor Stab LE Sweep [deg]</t>
+  </si>
+  <si>
+    <t>Max Mach at 30k ft</t>
   </si>
 </sst>
 </file>
@@ -871,7 +883,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2919600B-FD59-4F7A-AAA3-223AE9D885EC}">
-  <dimension ref="A1:L62"/>
+  <dimension ref="A1:L66"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="38.77734375" customWidth="1"/>
@@ -1281,7 +1293,7 @@
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A23" s="5" t="s">
-        <v>6</v>
+        <v>96</v>
       </c>
       <c r="B23" s="11"/>
       <c r="C23" s="11"/>
@@ -1293,47 +1305,45 @@
       <c r="I23" s="12"/>
       <c r="J23" s="12"/>
       <c r="K23" s="12"/>
-      <c r="L23" s="9" t="s">
+      <c r="L23" s="9"/>
+    </row>
+    <row r="24" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A24" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B24" s="11"/>
+      <c r="C24" s="11"/>
+      <c r="D24" s="11"/>
+      <c r="E24" s="11"/>
+      <c r="F24" s="12"/>
+      <c r="G24" s="12"/>
+      <c r="H24" s="12"/>
+      <c r="I24" s="12"/>
+      <c r="J24" s="12"/>
+      <c r="K24" s="12"/>
+      <c r="L24" s="9" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A24" s="4" t="s">
+    <row r="25" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A25" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="B24" s="15"/>
-      <c r="C24" s="15"/>
-      <c r="D24" s="15"/>
-      <c r="E24" s="15"/>
-      <c r="F24" s="15"/>
-      <c r="G24" s="15"/>
-      <c r="H24" s="15"/>
-      <c r="I24" s="15"/>
-      <c r="J24" s="15"/>
-      <c r="K24" s="15"/>
-      <c r="L24" s="10"/>
-    </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A25" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B25" s="11"/>
-      <c r="C25" s="11"/>
-      <c r="D25" s="11"/>
-      <c r="E25" s="11"/>
-      <c r="F25" s="12"/>
-      <c r="G25" s="12"/>
-      <c r="H25" s="12"/>
-      <c r="I25" s="12"/>
-      <c r="J25" s="12"/>
-      <c r="K25" s="12"/>
-      <c r="L25" s="9" t="s">
-        <v>10</v>
-      </c>
+      <c r="B25" s="15"/>
+      <c r="C25" s="15"/>
+      <c r="D25" s="15"/>
+      <c r="E25" s="15"/>
+      <c r="F25" s="15"/>
+      <c r="G25" s="15"/>
+      <c r="H25" s="15"/>
+      <c r="I25" s="15"/>
+      <c r="J25" s="15"/>
+      <c r="K25" s="15"/>
+      <c r="L25" s="10"/>
     </row>
     <row r="26" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A26" s="5" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B26" s="11"/>
       <c r="C26" s="11"/>
@@ -1346,12 +1356,12 @@
       <c r="J26" s="12"/>
       <c r="K26" s="12"/>
       <c r="L26" s="9" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="27" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A27" s="5" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B27" s="11"/>
       <c r="C27" s="11"/>
@@ -1364,12 +1374,12 @@
       <c r="J27" s="12"/>
       <c r="K27" s="12"/>
       <c r="L27" s="9" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A28" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B28" s="11"/>
       <c r="C28" s="11"/>
@@ -1382,12 +1392,12 @@
       <c r="J28" s="12"/>
       <c r="K28" s="12"/>
       <c r="L28" s="9" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="29" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A29" s="5" t="s">
-        <v>44</v>
+        <v>15</v>
       </c>
       <c r="B29" s="11"/>
       <c r="C29" s="11"/>
@@ -1399,11 +1409,13 @@
       <c r="I29" s="12"/>
       <c r="J29" s="12"/>
       <c r="K29" s="12"/>
-      <c r="L29" s="9"/>
+      <c r="L29" s="9" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="30" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A30" s="5" t="s">
-        <v>25</v>
+        <v>44</v>
       </c>
       <c r="B30" s="11"/>
       <c r="C30" s="11"/>
@@ -1415,13 +1427,11 @@
       <c r="I30" s="12"/>
       <c r="J30" s="12"/>
       <c r="K30" s="12"/>
-      <c r="L30" s="9" t="s">
-        <v>26</v>
-      </c>
+      <c r="L30" s="9"/>
     </row>
     <row r="31" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A31" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B31" s="11"/>
       <c r="C31" s="11"/>
@@ -1433,11 +1443,13 @@
       <c r="I31" s="12"/>
       <c r="J31" s="12"/>
       <c r="K31" s="12"/>
-      <c r="L31" s="9"/>
+      <c r="L31" s="9" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="32" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A32" s="5" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="B32" s="11"/>
       <c r="C32" s="11"/>
@@ -1449,13 +1461,11 @@
       <c r="I32" s="12"/>
       <c r="J32" s="12"/>
       <c r="K32" s="12"/>
-      <c r="L32" s="9" t="s">
-        <v>19</v>
-      </c>
+      <c r="L32" s="9"/>
     </row>
     <row r="33" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A33" s="5" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B33" s="11"/>
       <c r="C33" s="11"/>
@@ -1468,12 +1478,12 @@
       <c r="J33" s="12"/>
       <c r="K33" s="12"/>
       <c r="L33" s="9" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="34" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A34" s="5" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B34" s="11"/>
       <c r="C34" s="11"/>
@@ -1485,11 +1495,13 @@
       <c r="I34" s="12"/>
       <c r="J34" s="12"/>
       <c r="K34" s="12"/>
-      <c r="L34" s="9"/>
+      <c r="L34" s="9" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="35" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A35" s="5" t="s">
-        <v>89</v>
+        <v>22</v>
       </c>
       <c r="B35" s="11"/>
       <c r="C35" s="11"/>
@@ -1505,7 +1517,7 @@
     </row>
     <row r="36" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A36" s="5" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B36" s="11"/>
       <c r="C36" s="11"/>
@@ -1521,7 +1533,7 @@
     </row>
     <row r="37" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A37" s="5" t="s">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="B37" s="11"/>
       <c r="C37" s="11"/>
@@ -1533,13 +1545,11 @@
       <c r="I37" s="12"/>
       <c r="J37" s="12"/>
       <c r="K37" s="12"/>
-      <c r="L37" s="9" t="s">
-        <v>61</v>
-      </c>
+      <c r="L37" s="9"/>
     </row>
     <row r="38" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A38" s="5" t="s">
-        <v>27</v>
+        <v>60</v>
       </c>
       <c r="B38" s="11"/>
       <c r="C38" s="11"/>
@@ -1552,12 +1562,12 @@
       <c r="J38" s="12"/>
       <c r="K38" s="12"/>
       <c r="L38" s="9" t="s">
-        <v>28</v>
+        <v>61</v>
       </c>
     </row>
     <row r="39" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A39" s="5" t="s">
-        <v>47</v>
+        <v>27</v>
       </c>
       <c r="B39" s="11"/>
       <c r="C39" s="11"/>
@@ -1569,79 +1579,81 @@
       <c r="I39" s="12"/>
       <c r="J39" s="12"/>
       <c r="K39" s="12"/>
-      <c r="L39" s="9"/>
+      <c r="L39" s="9" t="s">
+        <v>28</v>
+      </c>
     </row>
     <row r="40" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A40" s="4" t="s">
+      <c r="A40" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="B40" s="11"/>
+      <c r="C40" s="11"/>
+      <c r="D40" s="11"/>
+      <c r="E40" s="11"/>
+      <c r="F40" s="12"/>
+      <c r="G40" s="12"/>
+      <c r="H40" s="12"/>
+      <c r="I40" s="12"/>
+      <c r="J40" s="12"/>
+      <c r="K40" s="12"/>
+      <c r="L40" s="9"/>
+    </row>
+    <row r="41" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A41" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="B40" s="15"/>
-      <c r="C40" s="15"/>
-      <c r="D40" s="15"/>
-      <c r="E40" s="15"/>
-      <c r="F40" s="15"/>
-      <c r="G40" s="15"/>
-      <c r="H40" s="15"/>
-      <c r="I40" s="15"/>
-      <c r="J40" s="15"/>
-      <c r="K40" s="15"/>
-      <c r="L40" s="10"/>
-    </row>
-    <row r="41" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A41" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="B41" s="11"/>
-      <c r="C41" s="14"/>
-      <c r="D41" s="14"/>
-      <c r="E41" s="14"/>
-      <c r="F41" s="13"/>
-      <c r="G41" s="13"/>
-      <c r="H41" s="13"/>
-      <c r="I41" s="13"/>
-      <c r="J41" s="12"/>
-      <c r="K41" s="12"/>
-      <c r="L41" s="9" t="s">
-        <v>83</v>
-      </c>
+      <c r="B41" s="15"/>
+      <c r="C41" s="15"/>
+      <c r="D41" s="15"/>
+      <c r="E41" s="15"/>
+      <c r="F41" s="15"/>
+      <c r="G41" s="15"/>
+      <c r="H41" s="15"/>
+      <c r="I41" s="15"/>
+      <c r="J41" s="15"/>
+      <c r="K41" s="15"/>
+      <c r="L41" s="10"/>
     </row>
     <row r="42" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A42" s="5" t="s">
-        <v>17</v>
+        <v>48</v>
       </c>
       <c r="B42" s="11"/>
-      <c r="C42" s="11"/>
-      <c r="D42" s="11"/>
-      <c r="E42" s="11"/>
-      <c r="F42" s="12"/>
-      <c r="G42" s="12"/>
-      <c r="H42" s="12"/>
-      <c r="I42" s="12"/>
+      <c r="C42" s="14"/>
+      <c r="D42" s="14"/>
+      <c r="E42" s="14"/>
+      <c r="F42" s="13"/>
+      <c r="G42" s="13"/>
+      <c r="H42" s="13"/>
+      <c r="I42" s="13"/>
       <c r="J42" s="12"/>
       <c r="K42" s="12"/>
       <c r="L42" s="9" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="43" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A43" s="5" t="s">
-        <v>91</v>
+        <v>17</v>
       </c>
       <c r="B43" s="11"/>
-      <c r="C43" s="14"/>
-      <c r="D43" s="14"/>
-      <c r="E43" s="14"/>
-      <c r="F43" s="13"/>
-      <c r="G43" s="13"/>
-      <c r="H43" s="13"/>
-      <c r="I43" s="13"/>
+      <c r="C43" s="11"/>
+      <c r="D43" s="11"/>
+      <c r="E43" s="11"/>
+      <c r="F43" s="12"/>
+      <c r="G43" s="12"/>
+      <c r="H43" s="12"/>
+      <c r="I43" s="12"/>
       <c r="J43" s="12"/>
       <c r="K43" s="12"/>
-      <c r="L43" s="9"/>
+      <c r="L43" s="9" t="s">
+        <v>84</v>
+      </c>
     </row>
     <row r="44" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A44" s="5" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B44" s="11"/>
       <c r="C44" s="14"/>
@@ -1657,7 +1669,7 @@
     </row>
     <row r="45" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A45" s="5" t="s">
-        <v>85</v>
+        <v>92</v>
       </c>
       <c r="B45" s="11"/>
       <c r="C45" s="14"/>
@@ -1673,7 +1685,7 @@
     </row>
     <row r="46" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A46" s="5" t="s">
-        <v>86</v>
+        <v>93</v>
       </c>
       <c r="B46" s="11"/>
       <c r="C46" s="14"/>
@@ -1689,7 +1701,7 @@
     </row>
     <row r="47" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A47" s="5" t="s">
-        <v>45</v>
+        <v>94</v>
       </c>
       <c r="B47" s="11"/>
       <c r="C47" s="14"/>
@@ -1705,7 +1717,7 @@
     </row>
     <row r="48" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A48" s="5" t="s">
-        <v>46</v>
+        <v>95</v>
       </c>
       <c r="B48" s="11"/>
       <c r="C48" s="14"/>
@@ -1721,7 +1733,7 @@
     </row>
     <row r="49" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A49" s="5" t="s">
-        <v>50</v>
+        <v>85</v>
       </c>
       <c r="B49" s="11"/>
       <c r="C49" s="14"/>
@@ -1737,7 +1749,7 @@
     </row>
     <row r="50" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A50" s="5" t="s">
-        <v>49</v>
+        <v>86</v>
       </c>
       <c r="B50" s="11"/>
       <c r="C50" s="14"/>
@@ -1753,7 +1765,7 @@
     </row>
     <row r="51" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A51" s="5" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="B51" s="11"/>
       <c r="C51" s="14"/>
@@ -1768,42 +1780,40 @@
       <c r="L51" s="9"/>
     </row>
     <row r="52" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A52" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="B52" s="15"/>
-      <c r="C52" s="15"/>
-      <c r="D52" s="15"/>
-      <c r="E52" s="15"/>
-      <c r="F52" s="15"/>
-      <c r="G52" s="15"/>
-      <c r="H52" s="15"/>
-      <c r="I52" s="15"/>
-      <c r="J52" s="15"/>
-      <c r="K52" s="15"/>
-      <c r="L52" s="10"/>
+      <c r="A52" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="B52" s="11"/>
+      <c r="C52" s="14"/>
+      <c r="D52" s="14"/>
+      <c r="E52" s="14"/>
+      <c r="F52" s="13"/>
+      <c r="G52" s="13"/>
+      <c r="H52" s="13"/>
+      <c r="I52" s="13"/>
+      <c r="J52" s="12"/>
+      <c r="K52" s="12"/>
+      <c r="L52" s="9"/>
     </row>
     <row r="53" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A53" s="5" t="s">
-        <v>64</v>
+        <v>50</v>
       </c>
       <c r="B53" s="11"/>
-      <c r="C53" s="11"/>
-      <c r="D53" s="11"/>
-      <c r="E53" s="11"/>
-      <c r="F53" s="12"/>
-      <c r="G53" s="12"/>
-      <c r="H53" s="12"/>
-      <c r="I53" s="12"/>
+      <c r="C53" s="14"/>
+      <c r="D53" s="14"/>
+      <c r="E53" s="14"/>
+      <c r="F53" s="13"/>
+      <c r="G53" s="13"/>
+      <c r="H53" s="13"/>
+      <c r="I53" s="13"/>
       <c r="J53" s="12"/>
       <c r="K53" s="12"/>
-      <c r="L53" s="9" t="s">
-        <v>66</v>
-      </c>
+      <c r="L53" s="9"/>
     </row>
     <row r="54" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A54" s="5" t="s">
-        <v>65</v>
+        <v>49</v>
       </c>
       <c r="B54" s="11"/>
       <c r="C54" s="14"/>
@@ -1819,7 +1829,7 @@
     </row>
     <row r="55" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A55" s="5" t="s">
-        <v>67</v>
+        <v>51</v>
       </c>
       <c r="B55" s="11"/>
       <c r="C55" s="14"/>
@@ -1834,40 +1844,42 @@
       <c r="L55" s="9"/>
     </row>
     <row r="56" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A56" s="5" t="s">
-        <v>68</v>
-      </c>
-      <c r="B56" s="11"/>
-      <c r="C56" s="14"/>
-      <c r="D56" s="14"/>
-      <c r="E56" s="14"/>
-      <c r="F56" s="13"/>
-      <c r="G56" s="13"/>
-      <c r="H56" s="13"/>
-      <c r="I56" s="13"/>
-      <c r="J56" s="12"/>
-      <c r="K56" s="12"/>
-      <c r="L56" s="9"/>
+      <c r="A56" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="B56" s="15"/>
+      <c r="C56" s="15"/>
+      <c r="D56" s="15"/>
+      <c r="E56" s="15"/>
+      <c r="F56" s="15"/>
+      <c r="G56" s="15"/>
+      <c r="H56" s="15"/>
+      <c r="I56" s="15"/>
+      <c r="J56" s="15"/>
+      <c r="K56" s="15"/>
+      <c r="L56" s="10"/>
     </row>
     <row r="57" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A57" s="5" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="B57" s="11"/>
-      <c r="C57" s="14"/>
-      <c r="D57" s="14"/>
-      <c r="E57" s="14"/>
-      <c r="F57" s="13"/>
-      <c r="G57" s="13"/>
-      <c r="H57" s="13"/>
-      <c r="I57" s="13"/>
+      <c r="C57" s="11"/>
+      <c r="D57" s="11"/>
+      <c r="E57" s="11"/>
+      <c r="F57" s="12"/>
+      <c r="G57" s="12"/>
+      <c r="H57" s="12"/>
+      <c r="I57" s="12"/>
       <c r="J57" s="12"/>
       <c r="K57" s="12"/>
-      <c r="L57" s="9"/>
+      <c r="L57" s="9" t="s">
+        <v>66</v>
+      </c>
     </row>
     <row r="58" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A58" s="5" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="B58" s="11"/>
       <c r="C58" s="14"/>
@@ -1883,7 +1895,7 @@
     </row>
     <row r="59" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A59" s="5" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="B59" s="11"/>
       <c r="C59" s="14"/>
@@ -1899,7 +1911,7 @@
     </row>
     <row r="60" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A60" s="5" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="B60" s="11"/>
       <c r="C60" s="14"/>
@@ -1915,7 +1927,7 @@
     </row>
     <row r="61" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A61" s="5" t="s">
-        <v>87</v>
+        <v>69</v>
       </c>
       <c r="B61" s="11"/>
       <c r="C61" s="14"/>
@@ -1931,7 +1943,7 @@
     </row>
     <row r="62" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A62" s="5" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="B62" s="11"/>
       <c r="C62" s="14"/>
@@ -1945,6 +1957,70 @@
       <c r="K62" s="12"/>
       <c r="L62" s="9"/>
     </row>
+    <row r="63" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A63" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="B63" s="11"/>
+      <c r="C63" s="14"/>
+      <c r="D63" s="14"/>
+      <c r="E63" s="14"/>
+      <c r="F63" s="13"/>
+      <c r="G63" s="13"/>
+      <c r="H63" s="13"/>
+      <c r="I63" s="13"/>
+      <c r="J63" s="12"/>
+      <c r="K63" s="12"/>
+      <c r="L63" s="9"/>
+    </row>
+    <row r="64" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A64" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="B64" s="11"/>
+      <c r="C64" s="14"/>
+      <c r="D64" s="14"/>
+      <c r="E64" s="14"/>
+      <c r="F64" s="13"/>
+      <c r="G64" s="13"/>
+      <c r="H64" s="13"/>
+      <c r="I64" s="13"/>
+      <c r="J64" s="12"/>
+      <c r="K64" s="12"/>
+      <c r="L64" s="9"/>
+    </row>
+    <row r="65" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A65" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="B65" s="11"/>
+      <c r="C65" s="14"/>
+      <c r="D65" s="14"/>
+      <c r="E65" s="14"/>
+      <c r="F65" s="13"/>
+      <c r="G65" s="13"/>
+      <c r="H65" s="13"/>
+      <c r="I65" s="13"/>
+      <c r="J65" s="12"/>
+      <c r="K65" s="12"/>
+      <c r="L65" s="9"/>
+    </row>
+    <row r="66" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A66" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="B66" s="11"/>
+      <c r="C66" s="14"/>
+      <c r="D66" s="14"/>
+      <c r="E66" s="14"/>
+      <c r="F66" s="13"/>
+      <c r="G66" s="13"/>
+      <c r="H66" s="13"/>
+      <c r="I66" s="13"/>
+      <c r="J66" s="12"/>
+      <c r="K66" s="12"/>
+      <c r="L66" s="9"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -1952,6 +2028,16 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f38bd768-81b4-450c-b73d-1a8fa3ba2722">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -1960,7 +2046,7 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100841FCFF63B2DEE4FAB3ABDCB2B58E191" ma:contentTypeVersion="9" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="6537ae6c172b48d8001feb3057ef3193">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="f38bd768-81b4-450c-b73d-1a8fa3ba2722" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="e79d1da23033c2d9c1658a7b9c3763cb" ns2:_="">
     <xsd:import namespace="f38bd768-81b4-450c-b73d-1a8fa3ba2722"/>
@@ -2132,17 +2218,17 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f38bd768-81b4-450c-b73d-1a8fa3ba2722">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C5DB6742-085C-4A8F-8C68-EE166C6FD496}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="f38bd768-81b4-450c-b73d-1a8fa3ba2722"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9162A322-41FC-4C0D-9942-C36B749F2613}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
@@ -2150,7 +2236,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A0D3B35F-2651-4930-8D88-666C35501CF8}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2166,14 +2252,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C5DB6742-085C-4A8F-8C68-EE166C6FD496}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="f38bd768-81b4-450c-b73d-1a8fa3ba2722"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
connected backend variables between concept_control and planeObj. Added CG estimate (With a bug) working to debug.
</commit_message>
<xml_diff>
--- a/Sizing/concepts_tabulations_template.xlsx
+++ b/Sizing/concepts_tabulations_template.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfile\Documents\MyDocuments\CODING\GitWorkingDirectory\team10aiaa\Sizing\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\VonBe\Documents\MATLAB\team10aiaa\Sizing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A629E1F0-03BC-4697-A28C-E4EA34D468C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10147D07-8566-48D1-A48E-F3F2CBCC26F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="20928" windowHeight="12432" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Concepts" sheetId="2" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="112">
   <si>
     <t>Deliverable</t>
   </si>
@@ -327,6 +327,51 @@
   </si>
   <si>
     <t>Max Mach at 30k ft</t>
+  </si>
+  <si>
+    <t>PSC</t>
+  </si>
+  <si>
+    <t>X coor root LE wing</t>
+  </si>
+  <si>
+    <t>Hor Stab Root Chord</t>
+  </si>
+  <si>
+    <t>Hor Stab Span</t>
+  </si>
+  <si>
+    <t>X coor root LE Hor Stab</t>
+  </si>
+  <si>
+    <t>Strake root chord</t>
+  </si>
+  <si>
+    <t>Strake taper ratio</t>
+  </si>
+  <si>
+    <t>Strake span</t>
+  </si>
+  <si>
+    <t>X coor root LE Strake</t>
+  </si>
+  <si>
+    <t>Strake LE Sweep</t>
+  </si>
+  <si>
+    <t>Ver Stab Root Chord</t>
+  </si>
+  <si>
+    <t>Ver Stab Taper Ratio</t>
+  </si>
+  <si>
+    <t>Ver Stab Span</t>
+  </si>
+  <si>
+    <t>X coor root LE Ver Stab</t>
+  </si>
+  <si>
+    <t>Ver Stab LE Sweep</t>
   </si>
 </sst>
 </file>
@@ -384,7 +429,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -498,11 +543,24 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -548,6 +606,15 @@
     </xf>
     <xf numFmtId="2" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -883,21 +950,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2919600B-FD59-4F7A-AAA3-223AE9D885EC}">
-  <dimension ref="A1:L66"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:M89"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
-    <col min="1" max="1" width="38.77734375" customWidth="1"/>
-    <col min="2" max="2" width="10.44140625" customWidth="1"/>
-    <col min="3" max="3" width="12.44140625" customWidth="1"/>
-    <col min="4" max="5" width="4.6640625" customWidth="1"/>
-    <col min="6" max="8" width="9.77734375" customWidth="1"/>
-    <col min="9" max="9" width="10.44140625" customWidth="1"/>
-    <col min="10" max="10" width="9.77734375" customWidth="1"/>
-    <col min="11" max="11" width="10.44140625" customWidth="1"/>
-    <col min="12" max="12" width="106.77734375" customWidth="1"/>
+    <col min="1" max="1" width="38.7890625" customWidth="1"/>
+    <col min="2" max="2" width="10.41796875" customWidth="1"/>
+    <col min="3" max="3" width="12.41796875" customWidth="1"/>
+    <col min="4" max="5" width="4.68359375" customWidth="1"/>
+    <col min="6" max="8" width="9.7890625" customWidth="1"/>
+    <col min="9" max="9" width="10.41796875" customWidth="1"/>
+    <col min="10" max="10" width="9.7890625" customWidth="1"/>
+    <col min="11" max="12" width="10.41796875" customWidth="1"/>
+    <col min="13" max="13" width="106.7890625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:13" ht="14.7" thickBot="1" x14ac:dyDescent="0.6">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -931,11 +998,14 @@
       <c r="K1" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="L1" s="6" t="s">
+      <c r="L1" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="M1" s="6" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" s="2" t="s">
         <v>5</v>
       </c>
@@ -949,9 +1019,10 @@
       <c r="I2" s="3"/>
       <c r="J2" s="3"/>
       <c r="K2" s="3"/>
-      <c r="L2" s="7"/>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="L2" s="3"/>
+      <c r="M2" s="7"/>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" s="5" t="s">
         <v>56</v>
       </c>
@@ -965,11 +1036,12 @@
       <c r="I3" s="12"/>
       <c r="J3" s="13"/>
       <c r="K3" s="13"/>
-      <c r="L3" s="8" t="s">
+      <c r="L3" s="13"/>
+      <c r="M3" s="8" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="5" t="s">
         <v>58</v>
       </c>
@@ -983,11 +1055,12 @@
       <c r="I4" s="12"/>
       <c r="J4" s="13"/>
       <c r="K4" s="13"/>
-      <c r="L4" s="8" t="s">
+      <c r="L4" s="13"/>
+      <c r="M4" s="8" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="5" t="s">
         <v>31</v>
       </c>
@@ -1001,11 +1074,12 @@
       <c r="I5" s="12"/>
       <c r="J5" s="13"/>
       <c r="K5" s="13"/>
-      <c r="L5" s="8" t="s">
+      <c r="L5" s="13"/>
+      <c r="M5" s="8" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" s="5" t="s">
         <v>32</v>
       </c>
@@ -1019,11 +1093,12 @@
       <c r="I6" s="12"/>
       <c r="J6" s="13"/>
       <c r="K6" s="13"/>
-      <c r="L6" s="8" t="s">
+      <c r="L6" s="13"/>
+      <c r="M6" s="8" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" s="5" t="s">
         <v>29</v>
       </c>
@@ -1037,11 +1112,12 @@
       <c r="I7" s="12"/>
       <c r="J7" s="13"/>
       <c r="K7" s="13"/>
-      <c r="L7" s="8" t="s">
+      <c r="L7" s="13"/>
+      <c r="M7" s="8" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="5" t="s">
         <v>62</v>
       </c>
@@ -1055,11 +1131,12 @@
       <c r="I8" s="12"/>
       <c r="J8" s="13"/>
       <c r="K8" s="13"/>
-      <c r="L8" s="8" t="s">
+      <c r="L8" s="13"/>
+      <c r="M8" s="8" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" s="5" t="s">
         <v>34</v>
       </c>
@@ -1073,9 +1150,10 @@
       <c r="I9" s="12"/>
       <c r="J9" s="13"/>
       <c r="K9" s="13"/>
-      <c r="L9" s="8"/>
-    </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="L9" s="13"/>
+      <c r="M9" s="8"/>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" s="5" t="s">
         <v>35</v>
       </c>
@@ -1089,9 +1167,10 @@
       <c r="I10" s="12"/>
       <c r="J10" s="13"/>
       <c r="K10" s="13"/>
-      <c r="L10" s="8"/>
-    </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="L10" s="13"/>
+      <c r="M10" s="8"/>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" s="5" t="s">
         <v>74</v>
       </c>
@@ -1105,9 +1184,10 @@
       <c r="I11" s="12"/>
       <c r="J11" s="13"/>
       <c r="K11" s="13"/>
-      <c r="L11" s="8"/>
-    </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="L11" s="13"/>
+      <c r="M11" s="8"/>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" s="5" t="s">
         <v>36</v>
       </c>
@@ -1121,9 +1201,10 @@
       <c r="I12" s="12"/>
       <c r="J12" s="13"/>
       <c r="K12" s="13"/>
-      <c r="L12" s="8"/>
-    </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="L12" s="13"/>
+      <c r="M12" s="8"/>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" s="5" t="s">
         <v>72</v>
       </c>
@@ -1137,9 +1218,10 @@
       <c r="I13" s="12"/>
       <c r="J13" s="13"/>
       <c r="K13" s="13"/>
-      <c r="L13" s="8"/>
-    </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="L13" s="13"/>
+      <c r="M13" s="8"/>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" s="5" t="s">
         <v>54</v>
       </c>
@@ -1153,11 +1235,12 @@
       <c r="I14" s="12"/>
       <c r="J14" s="12"/>
       <c r="K14" s="12"/>
-      <c r="L14" s="9" t="s">
+      <c r="L14" s="12"/>
+      <c r="M14" s="9" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A15" s="5" t="s">
         <v>55</v>
       </c>
@@ -1171,11 +1254,12 @@
       <c r="I15" s="12"/>
       <c r="J15" s="12"/>
       <c r="K15" s="12"/>
-      <c r="L15" s="9" t="s">
+      <c r="L15" s="12"/>
+      <c r="M15" s="9" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="5" t="s">
         <v>80</v>
       </c>
@@ -1189,9 +1273,10 @@
       <c r="I16" s="12"/>
       <c r="J16" s="12"/>
       <c r="K16" s="12"/>
-      <c r="L16" s="9"/>
-    </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="L16" s="12"/>
+      <c r="M16" s="9"/>
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" s="5" t="s">
         <v>81</v>
       </c>
@@ -1205,9 +1290,10 @@
       <c r="I17" s="12"/>
       <c r="J17" s="12"/>
       <c r="K17" s="12"/>
-      <c r="L17" s="9"/>
-    </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="L17" s="12"/>
+      <c r="M17" s="9"/>
+    </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A18" s="5" t="s">
         <v>82</v>
       </c>
@@ -1221,9 +1307,10 @@
       <c r="I18" s="12"/>
       <c r="J18" s="12"/>
       <c r="K18" s="12"/>
-      <c r="L18" s="9"/>
-    </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="L18" s="12"/>
+      <c r="M18" s="9"/>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A19" s="5" t="s">
         <v>39</v>
       </c>
@@ -1237,9 +1324,10 @@
       <c r="I19" s="12"/>
       <c r="J19" s="12"/>
       <c r="K19" s="12"/>
-      <c r="L19" s="9"/>
-    </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="L19" s="12"/>
+      <c r="M19" s="9"/>
+    </row>
+    <row r="20" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A20" s="5" t="s">
         <v>40</v>
       </c>
@@ -1253,9 +1341,10 @@
       <c r="I20" s="12"/>
       <c r="J20" s="12"/>
       <c r="K20" s="12"/>
-      <c r="L20" s="9"/>
-    </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="L20" s="12"/>
+      <c r="M20" s="9"/>
+    </row>
+    <row r="21" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A21" s="5" t="s">
         <v>41</v>
       </c>
@@ -1269,11 +1358,12 @@
       <c r="I21" s="12"/>
       <c r="J21" s="12"/>
       <c r="K21" s="12"/>
-      <c r="L21" s="9" t="s">
+      <c r="L21" s="12"/>
+      <c r="M21" s="9" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A22" s="5" t="s">
         <v>53</v>
       </c>
@@ -1287,11 +1377,12 @@
       <c r="I22" s="12"/>
       <c r="J22" s="12"/>
       <c r="K22" s="12"/>
-      <c r="L22" s="9" t="s">
+      <c r="L22" s="12"/>
+      <c r="M22" s="9" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A23" s="5" t="s">
         <v>96</v>
       </c>
@@ -1305,9 +1396,10 @@
       <c r="I23" s="12"/>
       <c r="J23" s="12"/>
       <c r="K23" s="12"/>
-      <c r="L23" s="9"/>
-    </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="L23" s="12"/>
+      <c r="M23" s="9"/>
+    </row>
+    <row r="24" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A24" s="5" t="s">
         <v>6</v>
       </c>
@@ -1321,11 +1413,12 @@
       <c r="I24" s="12"/>
       <c r="J24" s="12"/>
       <c r="K24" s="12"/>
-      <c r="L24" s="9" t="s">
+      <c r="L24" s="12"/>
+      <c r="M24" s="9" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A25" s="4" t="s">
         <v>23</v>
       </c>
@@ -1339,9 +1432,10 @@
       <c r="I25" s="15"/>
       <c r="J25" s="15"/>
       <c r="K25" s="15"/>
-      <c r="L25" s="10"/>
-    </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="L25" s="15"/>
+      <c r="M25" s="10"/>
+    </row>
+    <row r="26" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A26" s="5" t="s">
         <v>9</v>
       </c>
@@ -1355,11 +1449,12 @@
       <c r="I26" s="12"/>
       <c r="J26" s="12"/>
       <c r="K26" s="12"/>
-      <c r="L26" s="9" t="s">
+      <c r="L26" s="12"/>
+      <c r="M26" s="9" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A27" s="5" t="s">
         <v>11</v>
       </c>
@@ -1373,11 +1468,12 @@
       <c r="I27" s="12"/>
       <c r="J27" s="12"/>
       <c r="K27" s="12"/>
-      <c r="L27" s="9" t="s">
+      <c r="L27" s="12"/>
+      <c r="M27" s="9" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A28" s="5" t="s">
         <v>13</v>
       </c>
@@ -1391,11 +1487,12 @@
       <c r="I28" s="12"/>
       <c r="J28" s="12"/>
       <c r="K28" s="12"/>
-      <c r="L28" s="9" t="s">
+      <c r="L28" s="12"/>
+      <c r="M28" s="9" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A29" s="5" t="s">
         <v>15</v>
       </c>
@@ -1409,11 +1506,12 @@
       <c r="I29" s="12"/>
       <c r="J29" s="12"/>
       <c r="K29" s="12"/>
-      <c r="L29" s="9" t="s">
+      <c r="L29" s="12"/>
+      <c r="M29" s="9" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A30" s="5" t="s">
         <v>44</v>
       </c>
@@ -1427,9 +1525,10 @@
       <c r="I30" s="12"/>
       <c r="J30" s="12"/>
       <c r="K30" s="12"/>
-      <c r="L30" s="9"/>
-    </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="L30" s="12"/>
+      <c r="M30" s="9"/>
+    </row>
+    <row r="31" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A31" s="5" t="s">
         <v>25</v>
       </c>
@@ -1443,11 +1542,12 @@
       <c r="I31" s="12"/>
       <c r="J31" s="12"/>
       <c r="K31" s="12"/>
-      <c r="L31" s="9" t="s">
+      <c r="L31" s="12"/>
+      <c r="M31" s="9" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A32" s="5" t="s">
         <v>24</v>
       </c>
@@ -1461,9 +1561,10 @@
       <c r="I32" s="12"/>
       <c r="J32" s="12"/>
       <c r="K32" s="12"/>
-      <c r="L32" s="9"/>
-    </row>
-    <row r="33" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="L32" s="12"/>
+      <c r="M32" s="9"/>
+    </row>
+    <row r="33" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A33" s="5" t="s">
         <v>18</v>
       </c>
@@ -1477,11 +1578,12 @@
       <c r="I33" s="12"/>
       <c r="J33" s="12"/>
       <c r="K33" s="12"/>
-      <c r="L33" s="9" t="s">
+      <c r="L33" s="12"/>
+      <c r="M33" s="9" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="34" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A34" s="5" t="s">
         <v>20</v>
       </c>
@@ -1495,11 +1597,12 @@
       <c r="I34" s="12"/>
       <c r="J34" s="12"/>
       <c r="K34" s="12"/>
-      <c r="L34" s="9" t="s">
+      <c r="L34" s="12"/>
+      <c r="M34" s="9" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="35" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A35" s="5" t="s">
         <v>22</v>
       </c>
@@ -1513,9 +1616,10 @@
       <c r="I35" s="12"/>
       <c r="J35" s="12"/>
       <c r="K35" s="12"/>
-      <c r="L35" s="9"/>
-    </row>
-    <row r="36" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="L35" s="12"/>
+      <c r="M35" s="9"/>
+    </row>
+    <row r="36" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A36" s="5" t="s">
         <v>89</v>
       </c>
@@ -1529,9 +1633,10 @@
       <c r="I36" s="12"/>
       <c r="J36" s="12"/>
       <c r="K36" s="12"/>
-      <c r="L36" s="9"/>
-    </row>
-    <row r="37" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="L36" s="12"/>
+      <c r="M36" s="9"/>
+    </row>
+    <row r="37" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A37" s="5" t="s">
         <v>90</v>
       </c>
@@ -1545,9 +1650,10 @@
       <c r="I37" s="12"/>
       <c r="J37" s="12"/>
       <c r="K37" s="12"/>
-      <c r="L37" s="9"/>
-    </row>
-    <row r="38" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="L37" s="12"/>
+      <c r="M37" s="9"/>
+    </row>
+    <row r="38" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A38" s="5" t="s">
         <v>60</v>
       </c>
@@ -1561,11 +1667,12 @@
       <c r="I38" s="12"/>
       <c r="J38" s="12"/>
       <c r="K38" s="12"/>
-      <c r="L38" s="9" t="s">
+      <c r="L38" s="12"/>
+      <c r="M38" s="9" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="39" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A39" s="5" t="s">
         <v>27</v>
       </c>
@@ -1579,12 +1686,13 @@
       <c r="I39" s="12"/>
       <c r="J39" s="12"/>
       <c r="K39" s="12"/>
-      <c r="L39" s="9" t="s">
+      <c r="L39" s="12"/>
+      <c r="M39" s="9" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="40" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A40" s="5" t="s">
+    <row r="40" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+      <c r="A40" s="17" t="s">
         <v>47</v>
       </c>
       <c r="B40" s="11"/>
@@ -1597,45 +1705,44 @@
       <c r="I40" s="12"/>
       <c r="J40" s="12"/>
       <c r="K40" s="12"/>
-      <c r="L40" s="9"/>
-    </row>
-    <row r="41" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A41" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="B41" s="15"/>
-      <c r="C41" s="15"/>
-      <c r="D41" s="15"/>
-      <c r="E41" s="15"/>
-      <c r="F41" s="15"/>
-      <c r="G41" s="15"/>
-      <c r="H41" s="15"/>
-      <c r="I41" s="15"/>
-      <c r="J41" s="15"/>
-      <c r="K41" s="15"/>
-      <c r="L41" s="10"/>
-    </row>
-    <row r="42" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A42" s="5" t="s">
-        <v>48</v>
+      <c r="L40" s="12"/>
+      <c r="M40" s="9"/>
+    </row>
+    <row r="41" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+      <c r="A41" s="16"/>
+      <c r="B41" s="11"/>
+      <c r="C41" s="11"/>
+      <c r="D41" s="11"/>
+      <c r="E41" s="11"/>
+      <c r="F41" s="12"/>
+      <c r="G41" s="12"/>
+      <c r="H41" s="12"/>
+      <c r="I41" s="12"/>
+      <c r="J41" s="12"/>
+      <c r="K41" s="12"/>
+      <c r="L41" s="12"/>
+      <c r="M41" s="9"/>
+    </row>
+    <row r="42" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+      <c r="A42" s="18" t="s">
+        <v>98</v>
       </c>
       <c r="B42" s="11"/>
-      <c r="C42" s="14"/>
-      <c r="D42" s="14"/>
-      <c r="E42" s="14"/>
-      <c r="F42" s="13"/>
-      <c r="G42" s="13"/>
-      <c r="H42" s="13"/>
-      <c r="I42" s="13"/>
+      <c r="C42" s="11"/>
+      <c r="D42" s="11"/>
+      <c r="E42" s="11"/>
+      <c r="F42" s="12"/>
+      <c r="G42" s="12"/>
+      <c r="H42" s="12"/>
+      <c r="I42" s="12"/>
       <c r="J42" s="12"/>
       <c r="K42" s="12"/>
-      <c r="L42" s="9" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="43" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A43" s="5" t="s">
-        <v>17</v>
+      <c r="L42" s="12"/>
+      <c r="M42" s="9"/>
+    </row>
+    <row r="43" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+      <c r="A43" s="18" t="s">
+        <v>101</v>
       </c>
       <c r="B43" s="11"/>
       <c r="C43" s="11"/>
@@ -1647,189 +1754,199 @@
       <c r="I43" s="12"/>
       <c r="J43" s="12"/>
       <c r="K43" s="12"/>
-      <c r="L43" s="9" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="44" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A44" s="5" t="s">
-        <v>91</v>
+      <c r="L43" s="12"/>
+      <c r="M43" s="9"/>
+    </row>
+    <row r="44" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+      <c r="A44" s="18" t="s">
+        <v>102</v>
       </c>
       <c r="B44" s="11"/>
-      <c r="C44" s="14"/>
-      <c r="D44" s="14"/>
-      <c r="E44" s="14"/>
-      <c r="F44" s="13"/>
-      <c r="G44" s="13"/>
-      <c r="H44" s="13"/>
-      <c r="I44" s="13"/>
+      <c r="C44" s="11"/>
+      <c r="D44" s="11"/>
+      <c r="E44" s="11"/>
+      <c r="F44" s="12"/>
+      <c r="G44" s="12"/>
+      <c r="H44" s="12"/>
+      <c r="I44" s="12"/>
       <c r="J44" s="12"/>
       <c r="K44" s="12"/>
-      <c r="L44" s="9"/>
-    </row>
-    <row r="45" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A45" s="5" t="s">
-        <v>92</v>
+      <c r="L44" s="12"/>
+      <c r="M44" s="9"/>
+    </row>
+    <row r="45" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+      <c r="A45" s="18" t="s">
+        <v>103</v>
       </c>
       <c r="B45" s="11"/>
-      <c r="C45" s="14"/>
-      <c r="D45" s="14"/>
-      <c r="E45" s="14"/>
-      <c r="F45" s="13"/>
-      <c r="G45" s="13"/>
-      <c r="H45" s="13"/>
-      <c r="I45" s="13"/>
+      <c r="C45" s="11"/>
+      <c r="D45" s="11"/>
+      <c r="E45" s="11"/>
+      <c r="F45" s="12"/>
+      <c r="G45" s="12"/>
+      <c r="H45" s="12"/>
+      <c r="I45" s="12"/>
       <c r="J45" s="12"/>
       <c r="K45" s="12"/>
-      <c r="L45" s="9"/>
-    </row>
-    <row r="46" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A46" s="5" t="s">
-        <v>93</v>
+      <c r="L45" s="12"/>
+      <c r="M45" s="9"/>
+    </row>
+    <row r="46" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+      <c r="A46" s="18" t="s">
+        <v>104</v>
       </c>
       <c r="B46" s="11"/>
-      <c r="C46" s="14"/>
-      <c r="D46" s="14"/>
-      <c r="E46" s="14"/>
-      <c r="F46" s="13"/>
-      <c r="G46" s="13"/>
-      <c r="H46" s="13"/>
-      <c r="I46" s="13"/>
+      <c r="C46" s="11"/>
+      <c r="D46" s="11"/>
+      <c r="E46" s="11"/>
+      <c r="F46" s="12"/>
+      <c r="G46" s="12"/>
+      <c r="H46" s="12"/>
+      <c r="I46" s="12"/>
       <c r="J46" s="12"/>
       <c r="K46" s="12"/>
-      <c r="L46" s="9"/>
-    </row>
-    <row r="47" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A47" s="5" t="s">
-        <v>94</v>
+      <c r="L46" s="12"/>
+      <c r="M46" s="9"/>
+    </row>
+    <row r="47" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+      <c r="A47" s="18" t="s">
+        <v>105</v>
       </c>
       <c r="B47" s="11"/>
-      <c r="C47" s="14"/>
-      <c r="D47" s="14"/>
-      <c r="E47" s="14"/>
-      <c r="F47" s="13"/>
-      <c r="G47" s="13"/>
-      <c r="H47" s="13"/>
-      <c r="I47" s="13"/>
+      <c r="C47" s="11"/>
+      <c r="D47" s="11"/>
+      <c r="E47" s="11"/>
+      <c r="F47" s="12"/>
+      <c r="G47" s="12"/>
+      <c r="H47" s="12"/>
+      <c r="I47" s="12"/>
       <c r="J47" s="12"/>
       <c r="K47" s="12"/>
-      <c r="L47" s="9"/>
-    </row>
-    <row r="48" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A48" s="5" t="s">
-        <v>95</v>
+      <c r="L47" s="12"/>
+      <c r="M47" s="9"/>
+    </row>
+    <row r="48" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+      <c r="A48" s="18" t="s">
+        <v>106</v>
       </c>
       <c r="B48" s="11"/>
-      <c r="C48" s="14"/>
-      <c r="D48" s="14"/>
-      <c r="E48" s="14"/>
-      <c r="F48" s="13"/>
-      <c r="G48" s="13"/>
-      <c r="H48" s="13"/>
-      <c r="I48" s="13"/>
+      <c r="C48" s="11"/>
+      <c r="D48" s="11"/>
+      <c r="E48" s="11"/>
+      <c r="F48" s="12"/>
+      <c r="G48" s="12"/>
+      <c r="H48" s="12"/>
+      <c r="I48" s="12"/>
       <c r="J48" s="12"/>
       <c r="K48" s="12"/>
-      <c r="L48" s="9"/>
-    </row>
-    <row r="49" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A49" s="5" t="s">
-        <v>85</v>
+      <c r="L48" s="12"/>
+      <c r="M48" s="9"/>
+    </row>
+    <row r="49" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+      <c r="A49" s="18" t="s">
+        <v>107</v>
       </c>
       <c r="B49" s="11"/>
-      <c r="C49" s="14"/>
-      <c r="D49" s="14"/>
-      <c r="E49" s="14"/>
-      <c r="F49" s="13"/>
-      <c r="G49" s="13"/>
-      <c r="H49" s="13"/>
-      <c r="I49" s="13"/>
+      <c r="C49" s="11"/>
+      <c r="D49" s="11"/>
+      <c r="E49" s="11"/>
+      <c r="F49" s="12"/>
+      <c r="G49" s="12"/>
+      <c r="H49" s="12"/>
+      <c r="I49" s="12"/>
       <c r="J49" s="12"/>
       <c r="K49" s="12"/>
-      <c r="L49" s="9"/>
-    </row>
-    <row r="50" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A50" s="5" t="s">
-        <v>86</v>
+      <c r="L49" s="12"/>
+      <c r="M49" s="9"/>
+    </row>
+    <row r="50" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+      <c r="A50" s="18" t="s">
+        <v>108</v>
       </c>
       <c r="B50" s="11"/>
-      <c r="C50" s="14"/>
-      <c r="D50" s="14"/>
-      <c r="E50" s="14"/>
-      <c r="F50" s="13"/>
-      <c r="G50" s="13"/>
-      <c r="H50" s="13"/>
-      <c r="I50" s="13"/>
+      <c r="C50" s="11"/>
+      <c r="D50" s="11"/>
+      <c r="E50" s="11"/>
+      <c r="F50" s="12"/>
+      <c r="G50" s="12"/>
+      <c r="H50" s="12"/>
+      <c r="I50" s="12"/>
       <c r="J50" s="12"/>
       <c r="K50" s="12"/>
-      <c r="L50" s="9"/>
-    </row>
-    <row r="51" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A51" s="5" t="s">
-        <v>45</v>
+      <c r="L50" s="12"/>
+      <c r="M50" s="9"/>
+    </row>
+    <row r="51" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+      <c r="A51" s="18" t="s">
+        <v>109</v>
       </c>
       <c r="B51" s="11"/>
-      <c r="C51" s="14"/>
-      <c r="D51" s="14"/>
-      <c r="E51" s="14"/>
-      <c r="F51" s="13"/>
-      <c r="G51" s="13"/>
-      <c r="H51" s="13"/>
-      <c r="I51" s="13"/>
+      <c r="C51" s="11"/>
+      <c r="D51" s="11"/>
+      <c r="E51" s="11"/>
+      <c r="F51" s="12"/>
+      <c r="G51" s="12"/>
+      <c r="H51" s="12"/>
+      <c r="I51" s="12"/>
       <c r="J51" s="12"/>
       <c r="K51" s="12"/>
-      <c r="L51" s="9"/>
-    </row>
-    <row r="52" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A52" s="5" t="s">
-        <v>46</v>
+      <c r="L51" s="12"/>
+      <c r="M51" s="9"/>
+    </row>
+    <row r="52" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+      <c r="A52" s="18" t="s">
+        <v>110</v>
       </c>
       <c r="B52" s="11"/>
-      <c r="C52" s="14"/>
-      <c r="D52" s="14"/>
-      <c r="E52" s="14"/>
-      <c r="F52" s="13"/>
-      <c r="G52" s="13"/>
-      <c r="H52" s="13"/>
-      <c r="I52" s="13"/>
+      <c r="C52" s="11"/>
+      <c r="D52" s="11"/>
+      <c r="E52" s="11"/>
+      <c r="F52" s="12"/>
+      <c r="G52" s="12"/>
+      <c r="H52" s="12"/>
+      <c r="I52" s="12"/>
       <c r="J52" s="12"/>
       <c r="K52" s="12"/>
-      <c r="L52" s="9"/>
-    </row>
-    <row r="53" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A53" s="5" t="s">
-        <v>50</v>
+      <c r="L52" s="12"/>
+      <c r="M52" s="9"/>
+    </row>
+    <row r="53" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+      <c r="A53" s="18" t="s">
+        <v>111</v>
       </c>
       <c r="B53" s="11"/>
-      <c r="C53" s="14"/>
-      <c r="D53" s="14"/>
-      <c r="E53" s="14"/>
-      <c r="F53" s="13"/>
-      <c r="G53" s="13"/>
-      <c r="H53" s="13"/>
-      <c r="I53" s="13"/>
+      <c r="C53" s="11"/>
+      <c r="D53" s="11"/>
+      <c r="E53" s="11"/>
+      <c r="F53" s="12"/>
+      <c r="G53" s="12"/>
+      <c r="H53" s="12"/>
+      <c r="I53" s="12"/>
       <c r="J53" s="12"/>
       <c r="K53" s="12"/>
-      <c r="L53" s="9"/>
-    </row>
-    <row r="54" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A54" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="B54" s="11"/>
-      <c r="C54" s="14"/>
-      <c r="D54" s="14"/>
-      <c r="E54" s="14"/>
-      <c r="F54" s="13"/>
-      <c r="G54" s="13"/>
-      <c r="H54" s="13"/>
-      <c r="I54" s="13"/>
-      <c r="J54" s="12"/>
-      <c r="K54" s="12"/>
-      <c r="L54" s="9"/>
-    </row>
-    <row r="55" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="L53" s="12"/>
+      <c r="M53" s="9"/>
+    </row>
+    <row r="54" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+      <c r="A54" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="B54" s="15"/>
+      <c r="C54" s="15"/>
+      <c r="D54" s="15"/>
+      <c r="E54" s="15"/>
+      <c r="F54" s="15"/>
+      <c r="G54" s="15"/>
+      <c r="H54" s="15"/>
+      <c r="I54" s="15"/>
+      <c r="J54" s="15"/>
+      <c r="K54" s="15"/>
+      <c r="L54" s="15"/>
+      <c r="M54" s="10"/>
+    </row>
+    <row r="55" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A55" s="5" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="B55" s="11"/>
       <c r="C55" s="14"/>
@@ -1841,45 +1958,50 @@
       <c r="I55" s="13"/>
       <c r="J55" s="12"/>
       <c r="K55" s="12"/>
-      <c r="L55" s="9"/>
-    </row>
-    <row r="56" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A56" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="B56" s="15"/>
-      <c r="C56" s="15"/>
-      <c r="D56" s="15"/>
-      <c r="E56" s="15"/>
-      <c r="F56" s="15"/>
-      <c r="G56" s="15"/>
-      <c r="H56" s="15"/>
-      <c r="I56" s="15"/>
-      <c r="J56" s="15"/>
-      <c r="K56" s="15"/>
-      <c r="L56" s="10"/>
-    </row>
-    <row r="57" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="L55" s="12"/>
+      <c r="M55" s="9" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="56" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+      <c r="A56" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="B56" s="11"/>
+      <c r="C56" s="11"/>
+      <c r="D56" s="11"/>
+      <c r="E56" s="11"/>
+      <c r="F56" s="12"/>
+      <c r="G56" s="12"/>
+      <c r="H56" s="12"/>
+      <c r="I56" s="12"/>
+      <c r="J56" s="12"/>
+      <c r="K56" s="12"/>
+      <c r="L56" s="12"/>
+      <c r="M56" s="9" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="57" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A57" s="5" t="s">
-        <v>64</v>
+        <v>91</v>
       </c>
       <c r="B57" s="11"/>
-      <c r="C57" s="11"/>
-      <c r="D57" s="11"/>
-      <c r="E57" s="11"/>
-      <c r="F57" s="12"/>
-      <c r="G57" s="12"/>
-      <c r="H57" s="12"/>
-      <c r="I57" s="12"/>
+      <c r="C57" s="14"/>
+      <c r="D57" s="14"/>
+      <c r="E57" s="14"/>
+      <c r="F57" s="13"/>
+      <c r="G57" s="13"/>
+      <c r="H57" s="13"/>
+      <c r="I57" s="13"/>
       <c r="J57" s="12"/>
       <c r="K57" s="12"/>
-      <c r="L57" s="9" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="58" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="L57" s="12"/>
+      <c r="M57" s="9"/>
+    </row>
+    <row r="58" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A58" s="5" t="s">
-        <v>65</v>
+        <v>92</v>
       </c>
       <c r="B58" s="11"/>
       <c r="C58" s="14"/>
@@ -1891,11 +2013,12 @@
       <c r="I58" s="13"/>
       <c r="J58" s="12"/>
       <c r="K58" s="12"/>
-      <c r="L58" s="9"/>
-    </row>
-    <row r="59" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="L58" s="12"/>
+      <c r="M58" s="9"/>
+    </row>
+    <row r="59" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A59" s="5" t="s">
-        <v>67</v>
+        <v>93</v>
       </c>
       <c r="B59" s="11"/>
       <c r="C59" s="14"/>
@@ -1907,11 +2030,12 @@
       <c r="I59" s="13"/>
       <c r="J59" s="12"/>
       <c r="K59" s="12"/>
-      <c r="L59" s="9"/>
-    </row>
-    <row r="60" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="L59" s="12"/>
+      <c r="M59" s="9"/>
+    </row>
+    <row r="60" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A60" s="5" t="s">
-        <v>68</v>
+        <v>94</v>
       </c>
       <c r="B60" s="11"/>
       <c r="C60" s="14"/>
@@ -1923,11 +2047,12 @@
       <c r="I60" s="13"/>
       <c r="J60" s="12"/>
       <c r="K60" s="12"/>
-      <c r="L60" s="9"/>
-    </row>
-    <row r="61" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="L60" s="12"/>
+      <c r="M60" s="9"/>
+    </row>
+    <row r="61" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A61" s="5" t="s">
-        <v>69</v>
+        <v>95</v>
       </c>
       <c r="B61" s="11"/>
       <c r="C61" s="14"/>
@@ -1939,11 +2064,12 @@
       <c r="I61" s="13"/>
       <c r="J61" s="12"/>
       <c r="K61" s="12"/>
-      <c r="L61" s="9"/>
-    </row>
-    <row r="62" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="L61" s="12"/>
+      <c r="M61" s="9"/>
+    </row>
+    <row r="62" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A62" s="5" t="s">
-        <v>70</v>
+        <v>85</v>
       </c>
       <c r="B62" s="11"/>
       <c r="C62" s="14"/>
@@ -1955,11 +2081,12 @@
       <c r="I62" s="13"/>
       <c r="J62" s="12"/>
       <c r="K62" s="12"/>
-      <c r="L62" s="9"/>
-    </row>
-    <row r="63" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="L62" s="12"/>
+      <c r="M62" s="9"/>
+    </row>
+    <row r="63" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A63" s="5" t="s">
-        <v>71</v>
+        <v>86</v>
       </c>
       <c r="B63" s="11"/>
       <c r="C63" s="14"/>
@@ -1971,11 +2098,12 @@
       <c r="I63" s="13"/>
       <c r="J63" s="12"/>
       <c r="K63" s="12"/>
-      <c r="L63" s="9"/>
-    </row>
-    <row r="64" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="L63" s="12"/>
+      <c r="M63" s="9"/>
+    </row>
+    <row r="64" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A64" s="5" t="s">
-        <v>73</v>
+        <v>45</v>
       </c>
       <c r="B64" s="11"/>
       <c r="C64" s="14"/>
@@ -1987,11 +2115,12 @@
       <c r="I64" s="13"/>
       <c r="J64" s="12"/>
       <c r="K64" s="12"/>
-      <c r="L64" s="9"/>
-    </row>
-    <row r="65" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="L64" s="12"/>
+      <c r="M64" s="9"/>
+    </row>
+    <row r="65" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A65" s="5" t="s">
-        <v>87</v>
+        <v>46</v>
       </c>
       <c r="B65" s="11"/>
       <c r="C65" s="14"/>
@@ -2003,11 +2132,12 @@
       <c r="I65" s="13"/>
       <c r="J65" s="12"/>
       <c r="K65" s="12"/>
-      <c r="L65" s="9"/>
-    </row>
-    <row r="66" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="L65" s="12"/>
+      <c r="M65" s="9"/>
+    </row>
+    <row r="66" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A66" s="5" t="s">
-        <v>88</v>
+        <v>50</v>
       </c>
       <c r="B66" s="11"/>
       <c r="C66" s="14"/>
@@ -2019,7 +2149,385 @@
       <c r="I66" s="13"/>
       <c r="J66" s="12"/>
       <c r="K66" s="12"/>
-      <c r="L66" s="9"/>
+      <c r="L66" s="12"/>
+      <c r="M66" s="9"/>
+    </row>
+    <row r="67" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+      <c r="A67" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="B67" s="11"/>
+      <c r="C67" s="14"/>
+      <c r="D67" s="14"/>
+      <c r="E67" s="14"/>
+      <c r="F67" s="13"/>
+      <c r="G67" s="13"/>
+      <c r="H67" s="13"/>
+      <c r="I67" s="13"/>
+      <c r="J67" s="12"/>
+      <c r="K67" s="12"/>
+      <c r="L67" s="12"/>
+      <c r="M67" s="9"/>
+    </row>
+    <row r="68" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+      <c r="A68" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="B68" s="11"/>
+      <c r="C68" s="14"/>
+      <c r="D68" s="14"/>
+      <c r="E68" s="14"/>
+      <c r="F68" s="13"/>
+      <c r="G68" s="13"/>
+      <c r="H68" s="13"/>
+      <c r="I68" s="13"/>
+      <c r="J68" s="12"/>
+      <c r="K68" s="12"/>
+      <c r="L68" s="12"/>
+      <c r="M68" s="9"/>
+    </row>
+    <row r="69" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+      <c r="A69" s="16" t="s">
+        <v>99</v>
+      </c>
+      <c r="B69" s="11"/>
+      <c r="C69" s="14"/>
+      <c r="D69" s="14"/>
+      <c r="E69" s="14"/>
+      <c r="F69" s="13"/>
+      <c r="G69" s="13"/>
+      <c r="H69" s="13"/>
+      <c r="I69" s="13"/>
+      <c r="J69" s="12"/>
+      <c r="K69" s="12"/>
+      <c r="L69" s="12"/>
+      <c r="M69" s="9"/>
+    </row>
+    <row r="70" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+      <c r="A70" s="16" t="s">
+        <v>100</v>
+      </c>
+      <c r="B70" s="11"/>
+      <c r="C70" s="14"/>
+      <c r="D70" s="14"/>
+      <c r="E70" s="14"/>
+      <c r="F70" s="13"/>
+      <c r="G70" s="13"/>
+      <c r="H70" s="13"/>
+      <c r="I70" s="13"/>
+      <c r="J70" s="12"/>
+      <c r="K70" s="12"/>
+      <c r="L70" s="12"/>
+      <c r="M70" s="9"/>
+    </row>
+    <row r="71" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+      <c r="A71" s="16"/>
+      <c r="B71" s="11"/>
+      <c r="C71" s="14"/>
+      <c r="D71" s="14"/>
+      <c r="E71" s="14"/>
+      <c r="F71" s="13"/>
+      <c r="G71" s="13"/>
+      <c r="H71" s="13"/>
+      <c r="I71" s="13"/>
+      <c r="J71" s="12"/>
+      <c r="K71" s="12"/>
+      <c r="L71" s="12"/>
+      <c r="M71" s="9"/>
+    </row>
+    <row r="72" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+      <c r="A72" s="16"/>
+      <c r="B72" s="11"/>
+      <c r="C72" s="14"/>
+      <c r="D72" s="14"/>
+      <c r="E72" s="14"/>
+      <c r="F72" s="13"/>
+      <c r="G72" s="13"/>
+      <c r="H72" s="13"/>
+      <c r="I72" s="13"/>
+      <c r="J72" s="12"/>
+      <c r="K72" s="12"/>
+      <c r="L72" s="12"/>
+      <c r="M72" s="9"/>
+    </row>
+    <row r="73" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+      <c r="A73" s="16"/>
+      <c r="B73" s="11"/>
+      <c r="C73" s="14"/>
+      <c r="D73" s="14"/>
+      <c r="E73" s="14"/>
+      <c r="F73" s="13"/>
+      <c r="G73" s="13"/>
+      <c r="H73" s="13"/>
+      <c r="I73" s="13"/>
+      <c r="J73" s="12"/>
+      <c r="K73" s="12"/>
+      <c r="L73" s="12"/>
+      <c r="M73" s="9"/>
+    </row>
+    <row r="74" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+      <c r="A74" s="16"/>
+      <c r="B74" s="11"/>
+      <c r="C74" s="14"/>
+      <c r="D74" s="14"/>
+      <c r="E74" s="14"/>
+      <c r="F74" s="13"/>
+      <c r="G74" s="13"/>
+      <c r="H74" s="13"/>
+      <c r="I74" s="13"/>
+      <c r="J74" s="12"/>
+      <c r="K74" s="12"/>
+      <c r="L74" s="12"/>
+      <c r="M74" s="9"/>
+    </row>
+    <row r="75" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+      <c r="A75" s="16"/>
+      <c r="B75" s="11"/>
+      <c r="C75" s="14"/>
+      <c r="D75" s="14"/>
+      <c r="E75" s="14"/>
+      <c r="F75" s="13"/>
+      <c r="G75" s="13"/>
+      <c r="H75" s="13"/>
+      <c r="I75" s="13"/>
+      <c r="J75" s="12"/>
+      <c r="K75" s="12"/>
+      <c r="L75" s="12"/>
+      <c r="M75" s="9"/>
+    </row>
+    <row r="76" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+      <c r="A76" s="16"/>
+      <c r="B76" s="11"/>
+      <c r="C76" s="14"/>
+      <c r="D76" s="14"/>
+      <c r="E76" s="14"/>
+      <c r="F76" s="13"/>
+      <c r="G76" s="13"/>
+      <c r="H76" s="13"/>
+      <c r="I76" s="13"/>
+      <c r="J76" s="12"/>
+      <c r="K76" s="12"/>
+      <c r="L76" s="12"/>
+      <c r="M76" s="9"/>
+    </row>
+    <row r="77" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+      <c r="A77" s="16"/>
+      <c r="B77" s="11"/>
+      <c r="C77" s="14"/>
+      <c r="D77" s="14"/>
+      <c r="E77" s="14"/>
+      <c r="F77" s="13"/>
+      <c r="G77" s="13"/>
+      <c r="H77" s="13"/>
+      <c r="I77" s="13"/>
+      <c r="J77" s="12"/>
+      <c r="K77" s="12"/>
+      <c r="L77" s="12"/>
+      <c r="M77" s="9"/>
+    </row>
+    <row r="78" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+      <c r="A78" s="16"/>
+      <c r="B78" s="11"/>
+      <c r="C78" s="14"/>
+      <c r="D78" s="14"/>
+      <c r="E78" s="14"/>
+      <c r="F78" s="13"/>
+      <c r="G78" s="13"/>
+      <c r="H78" s="13"/>
+      <c r="I78" s="13"/>
+      <c r="J78" s="12"/>
+      <c r="K78" s="12"/>
+      <c r="L78" s="12"/>
+      <c r="M78" s="9"/>
+    </row>
+    <row r="79" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+      <c r="A79" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="B79" s="15"/>
+      <c r="C79" s="15"/>
+      <c r="D79" s="15"/>
+      <c r="E79" s="15"/>
+      <c r="F79" s="15"/>
+      <c r="G79" s="15"/>
+      <c r="H79" s="15"/>
+      <c r="I79" s="15"/>
+      <c r="J79" s="15"/>
+      <c r="K79" s="15"/>
+      <c r="L79" s="15"/>
+      <c r="M79" s="10"/>
+    </row>
+    <row r="80" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+      <c r="A80" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="B80" s="11"/>
+      <c r="C80" s="11"/>
+      <c r="D80" s="11"/>
+      <c r="E80" s="11"/>
+      <c r="F80" s="12"/>
+      <c r="G80" s="12"/>
+      <c r="H80" s="12"/>
+      <c r="I80" s="12"/>
+      <c r="J80" s="12"/>
+      <c r="K80" s="12"/>
+      <c r="L80" s="12"/>
+      <c r="M80" s="9" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="81" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+      <c r="A81" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="B81" s="11"/>
+      <c r="C81" s="14"/>
+      <c r="D81" s="14"/>
+      <c r="E81" s="14"/>
+      <c r="F81" s="13"/>
+      <c r="G81" s="13"/>
+      <c r="H81" s="13"/>
+      <c r="I81" s="13"/>
+      <c r="J81" s="12"/>
+      <c r="K81" s="12"/>
+      <c r="L81" s="12"/>
+      <c r="M81" s="9"/>
+    </row>
+    <row r="82" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+      <c r="A82" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="B82" s="11"/>
+      <c r="C82" s="14"/>
+      <c r="D82" s="14"/>
+      <c r="E82" s="14"/>
+      <c r="F82" s="13"/>
+      <c r="G82" s="13"/>
+      <c r="H82" s="13"/>
+      <c r="I82" s="13"/>
+      <c r="J82" s="12"/>
+      <c r="K82" s="12"/>
+      <c r="L82" s="12"/>
+      <c r="M82" s="9"/>
+    </row>
+    <row r="83" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+      <c r="A83" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="B83" s="11"/>
+      <c r="C83" s="14"/>
+      <c r="D83" s="14"/>
+      <c r="E83" s="14"/>
+      <c r="F83" s="13"/>
+      <c r="G83" s="13"/>
+      <c r="H83" s="13"/>
+      <c r="I83" s="13"/>
+      <c r="J83" s="12"/>
+      <c r="K83" s="12"/>
+      <c r="L83" s="12"/>
+      <c r="M83" s="9"/>
+    </row>
+    <row r="84" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+      <c r="A84" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="B84" s="11"/>
+      <c r="C84" s="14"/>
+      <c r="D84" s="14"/>
+      <c r="E84" s="14"/>
+      <c r="F84" s="13"/>
+      <c r="G84" s="13"/>
+      <c r="H84" s="13"/>
+      <c r="I84" s="13"/>
+      <c r="J84" s="12"/>
+      <c r="K84" s="12"/>
+      <c r="L84" s="12"/>
+      <c r="M84" s="9"/>
+    </row>
+    <row r="85" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+      <c r="A85" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="B85" s="11"/>
+      <c r="C85" s="14"/>
+      <c r="D85" s="14"/>
+      <c r="E85" s="14"/>
+      <c r="F85" s="13"/>
+      <c r="G85" s="13"/>
+      <c r="H85" s="13"/>
+      <c r="I85" s="13"/>
+      <c r="J85" s="12"/>
+      <c r="K85" s="12"/>
+      <c r="L85" s="12"/>
+      <c r="M85" s="9"/>
+    </row>
+    <row r="86" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+      <c r="A86" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="B86" s="11"/>
+      <c r="C86" s="14"/>
+      <c r="D86" s="14"/>
+      <c r="E86" s="14"/>
+      <c r="F86" s="13"/>
+      <c r="G86" s="13"/>
+      <c r="H86" s="13"/>
+      <c r="I86" s="13"/>
+      <c r="J86" s="12"/>
+      <c r="K86" s="12"/>
+      <c r="L86" s="12"/>
+      <c r="M86" s="9"/>
+    </row>
+    <row r="87" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+      <c r="A87" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="B87" s="11"/>
+      <c r="C87" s="14"/>
+      <c r="D87" s="14"/>
+      <c r="E87" s="14"/>
+      <c r="F87" s="13"/>
+      <c r="G87" s="13"/>
+      <c r="H87" s="13"/>
+      <c r="I87" s="13"/>
+      <c r="J87" s="12"/>
+      <c r="K87" s="12"/>
+      <c r="L87" s="12"/>
+      <c r="M87" s="9"/>
+    </row>
+    <row r="88" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+      <c r="A88" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="B88" s="11"/>
+      <c r="C88" s="14"/>
+      <c r="D88" s="14"/>
+      <c r="E88" s="14"/>
+      <c r="F88" s="13"/>
+      <c r="G88" s="13"/>
+      <c r="H88" s="13"/>
+      <c r="I88" s="13"/>
+      <c r="J88" s="12"/>
+      <c r="K88" s="12"/>
+      <c r="L88" s="12"/>
+      <c r="M88" s="9"/>
+    </row>
+    <row r="89" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+      <c r="A89" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="B89" s="11"/>
+      <c r="C89" s="14"/>
+      <c r="D89" s="14"/>
+      <c r="E89" s="14"/>
+      <c r="F89" s="13"/>
+      <c r="G89" s="13"/>
+      <c r="H89" s="13"/>
+      <c r="I89" s="13"/>
+      <c r="J89" s="12"/>
+      <c r="K89" s="12"/>
+      <c r="L89" s="12"/>
+      <c r="M89" s="9"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2028,6 +2536,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="f38bd768-81b4-450c-b73d-1a8fa3ba2722">
@@ -2035,15 +2552,6 @@
     </lcf76f155ced4ddcb4097134ff3c332f>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2219,19 +2727,19 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9162A322-41FC-4C0D-9942-C36B749F2613}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C5DB6742-085C-4A8F-8C68-EE166C6FD496}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="f38bd768-81b4-450c-b73d-1a8fa3ba2722"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9162A322-41FC-4C0D-9942-C36B749F2613}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>